<commit_message>
complete uIR but no JP/MJP/QJP
</commit_message>
<xml_diff>
--- a/instructions.xlsx
+++ b/instructions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhjk/Sdu/COA/exp3_source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{310506AC-3709-A24A-AC12-F97436728669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3435E5C0-9810-DB4B-A00F-A0B32D113B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{F8C02137-E87E-3041-BB65-6214C9826856}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="150">
   <si>
     <t>微地址</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -571,10 +571,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>in-R0-2,IR,X,AR,DR</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>uIR[9]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -603,10 +599,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>out-R0-2,IR,Z,PC,DR</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>uIR[16]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -636,6 +628,14 @@
   </si>
   <si>
     <t>1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>o-R0-2,IR,Z,PC,DR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>i-R0-2,IR,X,AR,DR</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1057,22 +1057,22 @@
         <v>0</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>132</v>
@@ -1089,25 +1089,25 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>131</v>
@@ -1127,19 +1127,19 @@
         <v>113</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>97</v>
@@ -1156,19 +1156,19 @@
         <v>113</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>148</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>98</v>
@@ -1188,19 +1188,19 @@
         <v>113</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>94</v>
@@ -1222,19 +1222,19 @@
         <v>113</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>97</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>97</v>
@@ -1253,6 +1253,24 @@
       <c r="E8" s="2" t="s">
         <v>113</v>
       </c>
+      <c r="F8" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="10" spans="1:13">
       <c r="B10" s="2" t="s">
@@ -1264,6 +1282,24 @@
       <c r="E10" s="2" t="s">
         <v>113</v>
       </c>
+      <c r="F10" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="12" spans="1:13">
       <c r="B12" s="2" t="s">
@@ -1275,6 +1311,24 @@
       <c r="E12" s="2" t="s">
         <v>113</v>
       </c>
+      <c r="F12" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="14" spans="1:13">
       <c r="B14" s="2" t="s">
@@ -1286,6 +1340,24 @@
       <c r="E14" s="2" t="s">
         <v>113</v>
       </c>
+      <c r="F14" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
@@ -1302,8 +1374,26 @@
       <c r="E16" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="34">
+      <c r="F16" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="34">
       <c r="C17" s="1" t="s">
         <v>4</v>
       </c>
@@ -1313,8 +1403,26 @@
       <c r="E17" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
       <c r="C18" t="s">
         <v>20</v>
       </c>
@@ -1324,8 +1432,26 @@
       <c r="E18" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="17">
+      <c r="F18" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="17">
       <c r="B19" s="2" t="s">
         <v>14</v>
       </c>
@@ -1338,13 +1464,31 @@
       <c r="E19" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="17">
+    <row r="21" spans="1:11" ht="17">
       <c r="C21" s="1" t="s">
         <v>26</v>
       </c>
@@ -1354,8 +1498,26 @@
       <c r="E21" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="F21" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
       <c r="C22" t="s">
         <v>27</v>
       </c>
@@ -1365,8 +1527,26 @@
       <c r="E22" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="17">
+      <c r="F22" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="17">
       <c r="B23" s="2" t="s">
         <v>18</v>
       </c>
@@ -1379,13 +1559,31 @@
       <c r="E23" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="F23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
       <c r="A24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="17">
+    <row r="25" spans="1:11" ht="17">
       <c r="C25" s="1" t="s">
         <v>32</v>
       </c>
@@ -1395,8 +1593,26 @@
       <c r="E25" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="F25" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
       <c r="C26" t="s">
         <v>33</v>
       </c>
@@ -1406,8 +1622,26 @@
       <c r="E26" s="2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="17">
+      <c r="F26" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="17">
       <c r="B27" s="2" t="s">
         <v>18</v>
       </c>
@@ -1420,13 +1654,31 @@
       <c r="E27" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="F27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
       <c r="A28" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="17">
+    <row r="29" spans="1:11" ht="17">
       <c r="C29" s="1" t="s">
         <v>32</v>
       </c>
@@ -1436,8 +1688,26 @@
       <c r="E29" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="F29" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11">
       <c r="C30" t="s">
         <v>39</v>
       </c>
@@ -1447,8 +1717,26 @@
       <c r="E30" s="2" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="17">
+      <c r="F30" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="17">
       <c r="B31" s="2" t="s">
         <v>18</v>
       </c>
@@ -1461,13 +1749,31 @@
       <c r="E31" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="F31" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
       <c r="A32" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="17">
+    <row r="33" spans="1:11" ht="17">
       <c r="C33" s="1" t="s">
         <v>32</v>
       </c>
@@ -1477,8 +1783,26 @@
       <c r="E33" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="F33" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
       <c r="C34" t="s">
         <v>44</v>
       </c>
@@ -1488,8 +1812,26 @@
       <c r="E34" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="17">
+      <c r="F34" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="17">
       <c r="B35" s="2" t="s">
         <v>18</v>
       </c>
@@ -1502,13 +1844,31 @@
       <c r="E35" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="F35" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="17">
+    <row r="37" spans="1:11" ht="17">
       <c r="C37" s="1" t="s">
         <v>32</v>
       </c>
@@ -1518,8 +1878,26 @@
       <c r="E37" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="F37" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11">
       <c r="C38" t="s">
         <v>49</v>
       </c>
@@ -1529,8 +1907,26 @@
       <c r="E38" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="17">
+      <c r="F38" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="17">
       <c r="B39" s="2" t="s">
         <v>18</v>
       </c>
@@ -1543,13 +1939,31 @@
       <c r="E39" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="F39" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
       <c r="A40" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="17">
+    <row r="41" spans="1:11" ht="17">
       <c r="C41" s="1" t="s">
         <v>32</v>
       </c>
@@ -1559,8 +1973,26 @@
       <c r="E41" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="F41" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
       <c r="C42" t="s">
         <v>54</v>
       </c>
@@ -1570,8 +2002,26 @@
       <c r="E42" s="2" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" ht="17">
+      <c r="F42" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="17">
       <c r="B43" s="2" t="s">
         <v>18</v>
       </c>
@@ -1584,13 +2034,31 @@
       <c r="E43" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="F43" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11">
       <c r="A44" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="17">
+    <row r="45" spans="1:11" ht="17">
       <c r="C45" s="1" t="s">
         <v>32</v>
       </c>
@@ -1600,8 +2068,26 @@
       <c r="E45" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="46" spans="1:5">
+      <c r="F45" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11">
       <c r="C46" t="s">
         <v>59</v>
       </c>
@@ -1611,8 +2097,26 @@
       <c r="E46" s="2" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="17">
+      <c r="F46" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="17">
       <c r="B47" s="2" t="s">
         <v>18</v>
       </c>
@@ -1625,13 +2129,31 @@
       <c r="E47" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="48" spans="1:5">
+      <c r="F47" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11">
       <c r="A48" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="17">
+    <row r="49" spans="1:11" ht="17">
       <c r="C49" s="1" t="s">
         <v>32</v>
       </c>
@@ -1641,8 +2163,26 @@
       <c r="E49" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="50" spans="1:5">
+      <c r="F49" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11">
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -1652,8 +2192,26 @@
       <c r="E50" s="2" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" ht="17">
+      <c r="F50" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="17">
       <c r="B51" s="2" t="s">
         <v>18</v>
       </c>
@@ -1666,13 +2224,31 @@
       <c r="E51" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="52" spans="1:5">
+      <c r="F51" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11">
       <c r="A52" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="17">
+    <row r="53" spans="1:11" ht="17">
       <c r="C53" s="1" t="s">
         <v>32</v>
       </c>
@@ -1682,8 +2258,26 @@
       <c r="E53" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="54" spans="1:5">
+      <c r="F53" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11">
       <c r="C54" t="s">
         <v>68</v>
       </c>
@@ -1693,8 +2287,26 @@
       <c r="E54" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" ht="17">
+      <c r="F54" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="17">
       <c r="B55" s="2" t="s">
         <v>18</v>
       </c>
@@ -1707,13 +2319,31 @@
       <c r="E55" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="56" spans="1:5">
+      <c r="F55" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11">
       <c r="A56" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="17">
+    <row r="57" spans="1:11" ht="17">
       <c r="C57" s="1" t="s">
         <v>32</v>
       </c>
@@ -1723,8 +2353,26 @@
       <c r="E57" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="58" spans="1:5">
+      <c r="F57" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11">
       <c r="C58" t="s">
         <v>74</v>
       </c>
@@ -1734,8 +2382,26 @@
       <c r="E58" s="2" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" ht="17">
+      <c r="F58" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="17">
       <c r="B59" s="2" t="s">
         <v>18</v>
       </c>
@@ -1748,13 +2414,31 @@
       <c r="E59" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="60" spans="1:5">
+      <c r="F59" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11">
       <c r="A60" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="17">
+    <row r="61" spans="1:11" ht="17">
       <c r="C61" s="1" t="s">
         <v>32</v>
       </c>
@@ -1764,8 +2448,26 @@
       <c r="E61" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="62" spans="1:5">
+      <c r="F61" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11">
       <c r="C62" t="s">
         <v>79</v>
       </c>
@@ -1775,8 +2477,26 @@
       <c r="E62" s="2" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" ht="17">
+      <c r="F62" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="17">
       <c r="B63" s="2" t="s">
         <v>18</v>
       </c>
@@ -1789,13 +2509,31 @@
       <c r="E63" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="64" spans="1:5">
+      <c r="F63" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11">
       <c r="A64" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="17">
+    <row r="65" spans="1:11" ht="17">
       <c r="C65" s="1" t="s">
         <v>32</v>
       </c>
@@ -1805,8 +2543,26 @@
       <c r="E65" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="66" spans="1:5">
+      <c r="F65" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11">
       <c r="C66" t="s">
         <v>84</v>
       </c>
@@ -1816,8 +2572,26 @@
       <c r="E66" s="2" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" ht="17">
+      <c r="F66" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="17">
       <c r="B67" s="2" t="s">
         <v>18</v>
       </c>
@@ -1830,13 +2604,31 @@
       <c r="E67" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="68" spans="1:5">
+      <c r="F67" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11">
       <c r="A68" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="17">
+    <row r="69" spans="1:11" ht="17">
       <c r="B69" s="2" t="s">
         <v>18</v>
       </c>
@@ -1846,13 +2638,34 @@
       <c r="D69" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="70" spans="1:5">
+      <c r="E69" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11">
       <c r="A70" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="17">
+    <row r="71" spans="1:11" ht="17">
       <c r="C71" s="1" t="s">
         <v>32</v>
       </c>
@@ -1862,8 +2675,26 @@
       <c r="E71" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="72" spans="1:5">
+      <c r="F71" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J71" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K71" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11">
       <c r="C72" t="s">
         <v>92</v>
       </c>
@@ -1873,8 +2704,26 @@
       <c r="E72" s="2" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" ht="17">
+      <c r="F72" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K72" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="17">
       <c r="B73" s="2" t="s">
         <v>18</v>
       </c>
@@ -1887,13 +2736,31 @@
       <c r="E73" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="74" spans="1:5">
+      <c r="F73" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K73" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11">
       <c r="A74" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="17">
+    <row r="75" spans="1:11" ht="17">
       <c r="C75" s="1" t="s">
         <v>32</v>
       </c>
@@ -1903,8 +2770,26 @@
       <c r="E75" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="76" spans="1:5">
+      <c r="F75" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K75" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11">
       <c r="C76" t="s">
         <v>69</v>
       </c>
@@ -1914,8 +2799,26 @@
       <c r="E76" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" ht="17">
+      <c r="F76" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I76" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="17">
       <c r="B77" s="2" t="s">
         <v>18</v>
       </c>
@@ -1928,13 +2831,31 @@
       <c r="E77" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="78" spans="1:5">
+      <c r="F77" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H77" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K77" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11">
       <c r="A78" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="17">
+    <row r="79" spans="1:11" ht="17">
       <c r="C79" s="1" t="s">
         <v>32</v>
       </c>
@@ -1944,8 +2865,26 @@
       <c r="E79" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="80" spans="1:5">
+      <c r="F79" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K79" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11">
       <c r="C80" t="s">
         <v>68</v>
       </c>
@@ -1955,8 +2894,26 @@
       <c r="E80" s="2" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" ht="17">
+      <c r="F80" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="J80" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K80" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="17">
       <c r="B81" s="2" t="s">
         <v>18</v>
       </c>
@@ -1969,13 +2926,31 @@
       <c r="E81" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="82" spans="1:5">
+      <c r="F81" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J81" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K81" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11">
       <c r="A82" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="17">
+    <row r="83" spans="1:11" ht="17">
       <c r="C83" s="1" t="s">
         <v>2</v>
       </c>
@@ -1985,8 +2960,26 @@
       <c r="E83" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" ht="34">
+      <c r="F83" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I83" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K83" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="34">
       <c r="C84" s="1" t="s">
         <v>4</v>
       </c>
@@ -1996,8 +2989,26 @@
       <c r="E84" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" ht="17">
+      <c r="F84" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="I84" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K84" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" ht="17">
       <c r="B85" s="2" t="s">
         <v>18</v>
       </c>
@@ -2010,13 +3021,31 @@
       <c r="E85" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="86" spans="1:5">
+      <c r="F85" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I85" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="K85" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11">
       <c r="A86" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="17">
+    <row r="87" spans="1:11" ht="17">
       <c r="C87" s="1" t="s">
         <v>110</v>
       </c>

</xml_diff>

<commit_message>
convert bin to hex
</commit_message>
<xml_diff>
--- a/instructions.xlsx
+++ b/instructions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhjk/Sdu/COA/exp3_source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3435E5C0-9810-DB4B-A00F-A0B32D113B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7CC80A-8348-3F4A-97B9-AA46BF1E73D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{F8C02137-E87E-3041-BB65-6214C9826856}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="184">
   <si>
     <t>微地址</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -636,6 +636,142 @@
   </si>
   <si>
     <t>i-R0-2,IR,X,AR,DR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MDR-&gt;M(MAR)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>018</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>019</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>01A</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000000010011101</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000110000011000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000001000000010100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000001000000000100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000001000000001000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000001000000001100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000001000000011000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000000000100001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000011000011000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000001000100000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000001000000000010</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000001000010100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>001000010001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000101000000100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>001010010001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>001100010001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>001110010001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>010000000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>010010000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>010100000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>010110000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>111000000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>111010000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>111100000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000000010000000100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>100000000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>100010000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>100100000001000000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>000001000000010000</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1043,10 +1179,12 @@
     <col min="2" max="2" width="10.83203125" style="2"/>
     <col min="3" max="3" width="32.5" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" style="2" customWidth="1"/>
-    <col min="5" max="18" width="10.83203125" style="2"/>
+    <col min="5" max="13" width="10.83203125" style="2"/>
+    <col min="14" max="14" width="21.5" style="2" customWidth="1"/>
+    <col min="15" max="18" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="B1" s="2" t="s">
         <v>112</v>
       </c>
@@ -1084,7 +1222,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1116,7 +1254,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:14">
       <c r="C3" t="s">
         <v>2</v>
       </c>
@@ -1144,8 +1282,14 @@
       <c r="K3" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="32" customHeight="1">
+      <c r="L3" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="32" customHeight="1">
       <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1173,8 +1317,14 @@
       <c r="K4" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="L4" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
@@ -1205,13 +1355,19 @@
       <c r="K5" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="6" spans="1:13">
+      <c r="L5" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:14">
       <c r="C7" t="s">
         <v>2</v>
       </c>
@@ -1239,8 +1395,14 @@
       <c r="K7" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="34">
+      <c r="L7" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="34">
       <c r="B8" s="2" t="s">
         <v>14</v>
       </c>
@@ -1271,14 +1433,23 @@
       <c r="K8" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="10" spans="1:13">
+      <c r="L8" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="B10" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
       </c>
+      <c r="D10" s="2" t="s">
+        <v>152</v>
+      </c>
       <c r="E10" s="2" t="s">
         <v>113</v>
       </c>
@@ -1300,14 +1471,23 @@
       <c r="K10" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:13">
+      <c r="L10" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="B12" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C12" t="s">
         <v>16</v>
       </c>
+      <c r="D12" s="2" t="s">
+        <v>153</v>
+      </c>
       <c r="E12" s="2" t="s">
         <v>113</v>
       </c>
@@ -1329,14 +1509,23 @@
       <c r="K12" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:13">
+      <c r="L12" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="B14" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C14" t="s">
         <v>17</v>
       </c>
+      <c r="D14" s="2" t="s">
+        <v>154</v>
+      </c>
       <c r="E14" s="2" t="s">
         <v>113</v>
       </c>
@@ -1358,13 +1547,19 @@
       <c r="K14" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:13">
+      <c r="L14" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:14">
       <c r="C16" t="s">
         <v>2</v>
       </c>
@@ -1392,8 +1587,14 @@
       <c r="K16" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="34">
+      <c r="L16" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="34">
       <c r="C17" s="1" t="s">
         <v>4</v>
       </c>
@@ -1421,8 +1622,14 @@
       <c r="K17" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="18" spans="1:11">
+      <c r="L17" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
       <c r="C18" t="s">
         <v>20</v>
       </c>
@@ -1450,8 +1657,14 @@
       <c r="K18" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="17">
+      <c r="L18" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="17">
       <c r="B19" s="2" t="s">
         <v>14</v>
       </c>
@@ -1482,13 +1695,19 @@
       <c r="K19" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="20" spans="1:11">
+      <c r="L19" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="17">
+    <row r="21" spans="1:14" ht="17">
       <c r="C21" s="1" t="s">
         <v>26</v>
       </c>
@@ -1516,8 +1735,14 @@
       <c r="K21" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="22" spans="1:11">
+      <c r="L21" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
       <c r="C22" t="s">
         <v>27</v>
       </c>
@@ -1545,13 +1770,19 @@
       <c r="K22" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" ht="17">
+      <c r="L22" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="17">
       <c r="B23" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>3</v>
+        <v>151</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>30</v>
@@ -1560,7 +1791,7 @@
         <v>113</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>7</v>
@@ -1572,18 +1803,24 @@
         <v>144</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="24" spans="1:11">
+      <c r="L23" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="17">
+    <row r="25" spans="1:14" ht="17">
       <c r="C25" s="1" t="s">
         <v>32</v>
       </c>
@@ -1611,8 +1848,14 @@
       <c r="K25" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="26" spans="1:11">
+      <c r="L25" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
       <c r="C26" t="s">
         <v>33</v>
       </c>
@@ -1640,8 +1883,14 @@
       <c r="K26" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" ht="17">
+      <c r="L26" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="17">
       <c r="B27" s="2" t="s">
         <v>18</v>
       </c>
@@ -1672,13 +1921,19 @@
       <c r="K27" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="1:11">
+      <c r="L27" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="17">
+    <row r="29" spans="1:14" ht="17">
       <c r="C29" s="1" t="s">
         <v>32</v>
       </c>
@@ -1706,8 +1961,14 @@
       <c r="K29" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="30" spans="1:11">
+      <c r="L29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
       <c r="C30" t="s">
         <v>39</v>
       </c>
@@ -1735,8 +1996,14 @@
       <c r="K30" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" ht="17">
+      <c r="L30" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="17">
       <c r="B31" s="2" t="s">
         <v>18</v>
       </c>
@@ -1767,13 +2034,19 @@
       <c r="K31" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="32" spans="1:11">
+      <c r="L31" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="17">
+    <row r="33" spans="1:14" ht="17">
       <c r="C33" s="1" t="s">
         <v>32</v>
       </c>
@@ -1801,8 +2074,14 @@
       <c r="K33" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="34" spans="1:11">
+      <c r="L33" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
       <c r="C34" t="s">
         <v>44</v>
       </c>
@@ -1830,8 +2109,14 @@
       <c r="K34" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" ht="17">
+      <c r="L34" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="17">
       <c r="B35" s="2" t="s">
         <v>18</v>
       </c>
@@ -1862,13 +2147,19 @@
       <c r="K35" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:11">
+      <c r="L35" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="17">
+    <row r="37" spans="1:14" ht="17">
       <c r="C37" s="1" t="s">
         <v>32</v>
       </c>
@@ -1896,8 +2187,14 @@
       <c r="K37" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="38" spans="1:11">
+      <c r="L37" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
       <c r="C38" t="s">
         <v>49</v>
       </c>
@@ -1925,8 +2222,14 @@
       <c r="K38" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" ht="17">
+      <c r="L38" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="17">
       <c r="B39" s="2" t="s">
         <v>18</v>
       </c>
@@ -1957,13 +2260,19 @@
       <c r="K39" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="1:11">
+      <c r="L39" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="17">
+    <row r="41" spans="1:14" ht="17">
       <c r="C41" s="1" t="s">
         <v>32</v>
       </c>
@@ -1991,8 +2300,14 @@
       <c r="K41" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="42" spans="1:11">
+      <c r="L41" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
       <c r="C42" t="s">
         <v>54</v>
       </c>
@@ -2020,8 +2335,14 @@
       <c r="K42" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" ht="17">
+      <c r="L42" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="17">
       <c r="B43" s="2" t="s">
         <v>18</v>
       </c>
@@ -2052,13 +2373,19 @@
       <c r="K43" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="44" spans="1:11">
+      <c r="L43" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
       <c r="A44" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="17">
+    <row r="45" spans="1:14" ht="17">
       <c r="C45" s="1" t="s">
         <v>32</v>
       </c>
@@ -2086,8 +2413,14 @@
       <c r="K45" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="46" spans="1:11">
+      <c r="L45" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
       <c r="C46" t="s">
         <v>59</v>
       </c>
@@ -2115,8 +2448,14 @@
       <c r="K46" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" ht="17">
+      <c r="L46" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="17">
       <c r="B47" s="2" t="s">
         <v>18</v>
       </c>
@@ -2147,13 +2486,19 @@
       <c r="K47" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="48" spans="1:11">
+      <c r="L47" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N47" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
       <c r="A48" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="17">
+    <row r="49" spans="1:14" ht="17">
       <c r="C49" s="1" t="s">
         <v>32</v>
       </c>
@@ -2181,8 +2526,14 @@
       <c r="K49" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="50" spans="1:11">
+      <c r="L49" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14">
       <c r="C50" t="s">
         <v>69</v>
       </c>
@@ -2210,8 +2561,14 @@
       <c r="K50" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" ht="17">
+      <c r="L50" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="17">
       <c r="B51" s="2" t="s">
         <v>18</v>
       </c>
@@ -2242,13 +2599,19 @@
       <c r="K51" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="52" spans="1:11">
+      <c r="L51" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14">
       <c r="A52" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="17">
+    <row r="53" spans="1:14" ht="17">
       <c r="C53" s="1" t="s">
         <v>32</v>
       </c>
@@ -2276,8 +2639,14 @@
       <c r="K53" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="54" spans="1:11">
+      <c r="L53" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
       <c r="C54" t="s">
         <v>68</v>
       </c>
@@ -2305,8 +2674,14 @@
       <c r="K54" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" ht="17">
+      <c r="L54" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" ht="17">
       <c r="B55" s="2" t="s">
         <v>18</v>
       </c>
@@ -2337,13 +2712,19 @@
       <c r="K55" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="56" spans="1:11">
+      <c r="L55" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
       <c r="A56" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="17">
+    <row r="57" spans="1:14" ht="17">
       <c r="C57" s="1" t="s">
         <v>32</v>
       </c>
@@ -2371,8 +2752,14 @@
       <c r="K57" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="58" spans="1:11">
+      <c r="L57" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
       <c r="C58" t="s">
         <v>74</v>
       </c>
@@ -2400,8 +2787,14 @@
       <c r="K58" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" ht="17">
+      <c r="L58" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" ht="17">
       <c r="B59" s="2" t="s">
         <v>18</v>
       </c>
@@ -2432,13 +2825,19 @@
       <c r="K59" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="60" spans="1:11">
+      <c r="L59" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
       <c r="A60" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="17">
+    <row r="61" spans="1:14" ht="17">
       <c r="C61" s="1" t="s">
         <v>32</v>
       </c>
@@ -2466,8 +2865,14 @@
       <c r="K61" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="62" spans="1:11">
+      <c r="L61" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
       <c r="C62" t="s">
         <v>79</v>
       </c>
@@ -2495,8 +2900,14 @@
       <c r="K62" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" ht="17">
+      <c r="L62" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N62" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="17">
       <c r="B63" s="2" t="s">
         <v>18</v>
       </c>
@@ -2527,13 +2938,19 @@
       <c r="K63" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="64" spans="1:11">
+      <c r="L63" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N63" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14">
       <c r="A64" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="17">
+    <row r="65" spans="1:14" ht="17">
       <c r="C65" s="1" t="s">
         <v>32</v>
       </c>
@@ -2561,8 +2978,14 @@
       <c r="K65" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="66" spans="1:11">
+      <c r="L65" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N65" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
       <c r="C66" t="s">
         <v>84</v>
       </c>
@@ -2590,8 +3013,14 @@
       <c r="K66" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" ht="17">
+      <c r="L66" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N66" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" ht="17">
       <c r="B67" s="2" t="s">
         <v>18</v>
       </c>
@@ -2622,13 +3051,19 @@
       <c r="K67" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="68" spans="1:11">
+      <c r="L67" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N67" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
       <c r="A68" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="17">
+    <row r="69" spans="1:14" ht="17">
       <c r="B69" s="2" t="s">
         <v>18</v>
       </c>
@@ -2659,13 +3094,19 @@
       <c r="K69" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="1:11">
+      <c r="L69" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N69" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
       <c r="A70" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="17">
+    <row r="71" spans="1:14" ht="17">
       <c r="C71" s="1" t="s">
         <v>32</v>
       </c>
@@ -2693,8 +3134,14 @@
       <c r="K71" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="72" spans="1:11">
+      <c r="L71" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N71" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
       <c r="C72" t="s">
         <v>92</v>
       </c>
@@ -2722,8 +3169,14 @@
       <c r="K72" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" ht="17">
+      <c r="L72" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N72" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" ht="17">
       <c r="B73" s="2" t="s">
         <v>18</v>
       </c>
@@ -2754,13 +3207,19 @@
       <c r="K73" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="1:11">
+      <c r="L73" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N73" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
       <c r="A74" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="17">
+    <row r="75" spans="1:14" ht="17">
       <c r="C75" s="1" t="s">
         <v>32</v>
       </c>
@@ -2788,8 +3247,14 @@
       <c r="K75" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="76" spans="1:11">
+      <c r="L75" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N75" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
       <c r="C76" t="s">
         <v>69</v>
       </c>
@@ -2817,8 +3282,14 @@
       <c r="K76" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" ht="17">
+      <c r="L76" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N76" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" ht="17">
       <c r="B77" s="2" t="s">
         <v>18</v>
       </c>
@@ -2849,13 +3320,19 @@
       <c r="K77" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="78" spans="1:11">
+      <c r="L77" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N77" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14">
       <c r="A78" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="17">
+    <row r="79" spans="1:14" ht="17">
       <c r="C79" s="1" t="s">
         <v>32</v>
       </c>
@@ -2883,8 +3360,14 @@
       <c r="K79" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="80" spans="1:11">
+      <c r="L79" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N79" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14">
       <c r="C80" t="s">
         <v>68</v>
       </c>
@@ -2912,8 +3395,14 @@
       <c r="K80" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" ht="17">
+      <c r="L80" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N80" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" ht="17">
       <c r="B81" s="2" t="s">
         <v>18</v>
       </c>
@@ -2944,13 +3433,19 @@
       <c r="K81" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="82" spans="1:11">
+      <c r="L81" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N81" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14">
       <c r="A82" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="83" spans="1:11" ht="17">
+    <row r="83" spans="1:14" ht="17">
       <c r="C83" s="1" t="s">
         <v>2</v>
       </c>
@@ -2978,8 +3473,14 @@
       <c r="K83" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" ht="34">
+      <c r="L83" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N83" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" ht="34">
       <c r="C84" s="1" t="s">
         <v>4</v>
       </c>
@@ -3007,8 +3508,14 @@
       <c r="K84" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" ht="17">
+      <c r="L84" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="N84" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" ht="17">
       <c r="B85" s="2" t="s">
         <v>18</v>
       </c>
@@ -3039,13 +3546,19 @@
       <c r="K85" s="2" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="86" spans="1:11">
+      <c r="L85" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="N85" s="2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14">
       <c r="A86" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="87" spans="1:11" ht="17">
+    <row r="87" spans="1:14" ht="17">
       <c r="C87" s="1" t="s">
         <v>110</v>
       </c>

</xml_diff>